<commit_message>
đã fix lại import PC, HĐ, NKCT. test xuất ĐNTT word zip đã ok. test xuất ĐNTT excel cần sửa: KyThanhToan = tháng/năm tương ứng với kỳ can thiệp. Thêm ô chọn Người đề nghị (danh sách droplist gồm các CB có mã AVH)
</commit_message>
<xml_diff>
--- a/quanly/document_templates/thanh_toan_cong_can_thiep/Mau_DNTT.xlsx
+++ b/quanly/document_templates/thanh_toan_cong_can_thiep/Mau_DNTT.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dinht\source\repos\VietHealth.ContractManagement\VietHealth.ContractManagement\wwwroot\Templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\QLHD\quanly\document_templates\thanh_toan_cong_can_thiep\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{619B9B64-ABBB-4581-B44D-D7D8B1FC6238}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3BA58C8-1D82-4127-9044-454C4F4B15C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dia diem thuc hien" sheetId="5" r:id="rId1"/>
@@ -23,7 +23,7 @@
     <definedName name="List_CBNV">DataStaff[Họ và tên]</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">DNTT!$8:$11</definedName>
   </definedNames>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="108">
   <si>
     <t>ĐỀ NGHỊ THANH TOÁN</t>
   </si>
@@ -374,6 +374,9 @@
   </si>
   <si>
     <t>{{DiaDiemThucHien}}</t>
+  </si>
+  <si>
+    <t>Từ ngày {{TuNgay}} đến ngày {{DenNgay}}</t>
   </si>
 </sst>
 </file>
@@ -553,7 +556,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -598,6 +601,21 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -616,9 +634,6 @@
     <xf numFmtId="164" fontId="6" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -628,31 +643,12 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="4">
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <font>
         <b/>
@@ -684,6 +680,10 @@
           <color auto="1"/>
         </bottom>
       </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -728,7 +728,7 @@
   <autoFilter ref="A1:B27" xr:uid="{0128BF7A-BDDF-4535-96C6-8D2152CAEAE9}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{FFB1ECE8-3269-4708-AAE5-6BCCB211E6DF}" uniqueName="1" name="Nhóm HĐ" queryTableFieldId="1"/>
-    <tableColumn id="2" xr3:uid="{A707347A-9CCE-4F78-A5D7-AC3EA7DF8A95}" uniqueName="2" name="DDTH" queryTableFieldId="2" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{A707347A-9CCE-4F78-A5D7-AC3EA7DF8A95}" uniqueName="2" name="DDTH" queryTableFieldId="2" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -738,7 +738,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4A038C17-B4FC-4654-A744-93E1AF2ED608}" name="DataStaff" displayName="DataStaff" ref="A1:A28" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:A28" xr:uid="{4A038C17-B4FC-4654-A744-93E1AF2ED608}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{215A343C-297B-4885-ACC9-75826E986280}" uniqueName="1" name="Họ và tên" queryTableFieldId="1" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{215A343C-297B-4885-ACC9-75826E986280}" uniqueName="1" name="Họ và tên" queryTableFieldId="1" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1050,7 +1050,7 @@
       <c r="A2">
         <v>6</v>
       </c>
-      <c r="B2" s="34" t="s">
+      <c r="B2" t="s">
         <v>87</v>
       </c>
     </row>
@@ -1058,7 +1058,7 @@
       <c r="A3">
         <v>7</v>
       </c>
-      <c r="B3" s="34" t="s">
+      <c r="B3" t="s">
         <v>88</v>
       </c>
     </row>
@@ -1066,7 +1066,7 @@
       <c r="A4">
         <v>8</v>
       </c>
-      <c r="B4" s="34" t="s">
+      <c r="B4" t="s">
         <v>89</v>
       </c>
     </row>
@@ -1074,7 +1074,7 @@
       <c r="A5">
         <v>9</v>
       </c>
-      <c r="B5" s="34" t="s">
+      <c r="B5" t="s">
         <v>90</v>
       </c>
     </row>
@@ -1082,7 +1082,7 @@
       <c r="A6">
         <v>10</v>
       </c>
-      <c r="B6" s="34" t="s">
+      <c r="B6" t="s">
         <v>91</v>
       </c>
     </row>
@@ -1090,7 +1090,7 @@
       <c r="A7">
         <v>11</v>
       </c>
-      <c r="B7" s="34" t="s">
+      <c r="B7" t="s">
         <v>92</v>
       </c>
     </row>
@@ -1098,7 +1098,7 @@
       <c r="A8">
         <v>12</v>
       </c>
-      <c r="B8" s="34" t="s">
+      <c r="B8" t="s">
         <v>93</v>
       </c>
     </row>
@@ -1106,7 +1106,7 @@
       <c r="A9">
         <v>13</v>
       </c>
-      <c r="B9" s="34" t="s">
+      <c r="B9" t="s">
         <v>94</v>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       <c r="A10">
         <v>51</v>
       </c>
-      <c r="B10" s="34" t="s">
+      <c r="B10" t="s">
         <v>95</v>
       </c>
     </row>
@@ -1122,7 +1122,7 @@
       <c r="A11">
         <v>14</v>
       </c>
-      <c r="B11" s="34" t="s">
+      <c r="B11" t="s">
         <v>96</v>
       </c>
     </row>
@@ -1130,7 +1130,7 @@
       <c r="A12">
         <v>15</v>
       </c>
-      <c r="B12" s="34" t="s">
+      <c r="B12" t="s">
         <v>97</v>
       </c>
     </row>
@@ -1138,7 +1138,7 @@
       <c r="A13">
         <v>16</v>
       </c>
-      <c r="B13" s="34" t="s">
+      <c r="B13" t="s">
         <v>98</v>
       </c>
     </row>
@@ -1146,7 +1146,7 @@
       <c r="A14">
         <v>17</v>
       </c>
-      <c r="B14" s="34" t="s">
+      <c r="B14" t="s">
         <v>99</v>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       <c r="A15">
         <v>18</v>
       </c>
-      <c r="B15" s="34" t="s">
+      <c r="B15" t="s">
         <v>100</v>
       </c>
     </row>
@@ -1162,7 +1162,7 @@
       <c r="A16">
         <v>19</v>
       </c>
-      <c r="B16" s="34" t="s">
+      <c r="B16" t="s">
         <v>101</v>
       </c>
     </row>
@@ -1170,7 +1170,7 @@
       <c r="A17">
         <v>20</v>
       </c>
-      <c r="B17" s="34" t="s">
+      <c r="B17" t="s">
         <v>102</v>
       </c>
     </row>
@@ -1178,7 +1178,7 @@
       <c r="A18">
         <v>21</v>
       </c>
-      <c r="B18" s="34" t="s">
+      <c r="B18" t="s">
         <v>103</v>
       </c>
     </row>
@@ -1186,7 +1186,7 @@
       <c r="A19">
         <v>22</v>
       </c>
-      <c r="B19" s="34" t="s">
+      <c r="B19" t="s">
         <v>104</v>
       </c>
     </row>
@@ -1194,7 +1194,7 @@
       <c r="A20">
         <v>23</v>
       </c>
-      <c r="B20" s="34" t="s">
+      <c r="B20" t="s">
         <v>105</v>
       </c>
     </row>
@@ -1202,7 +1202,7 @@
       <c r="A21">
         <v>24</v>
       </c>
-      <c r="B21" s="34" t="s">
+      <c r="B21" t="s">
         <v>57</v>
       </c>
     </row>
@@ -1210,37 +1210,31 @@
       <c r="A22">
         <v>25</v>
       </c>
-      <c r="B22" s="34"/>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>26</v>
       </c>
-      <c r="B23" s="34"/>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>27</v>
       </c>
-      <c r="B24" s="34"/>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>28</v>
       </c>
-      <c r="B25" s="34"/>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>29</v>
       </c>
-      <c r="B26" s="34"/>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>30</v>
       </c>
-      <c r="B27" s="34"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1273,54 +1267,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
-      <c r="L1" s="20"/>
-      <c r="M1" s="20"/>
-      <c r="N1" s="20"/>
-      <c r="O1" s="20"/>
-      <c r="P1" s="20"/>
-      <c r="Q1" s="20"/>
-      <c r="R1" s="20"/>
-      <c r="S1" s="20"/>
-      <c r="T1" s="20"/>
-      <c r="U1" s="20"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+      <c r="K1" s="25"/>
+      <c r="L1" s="25"/>
+      <c r="M1" s="25"/>
+      <c r="N1" s="25"/>
+      <c r="O1" s="25"/>
+      <c r="P1" s="25"/>
+      <c r="Q1" s="25"/>
+      <c r="R1" s="25"/>
+      <c r="S1" s="25"/>
+      <c r="T1" s="25"/>
+      <c r="U1" s="25"/>
     </row>
     <row r="2" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="26" t="s">
         <v>55</v>
       </c>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
-      <c r="I2" s="21"/>
-      <c r="J2" s="21"/>
-      <c r="K2" s="21"/>
-      <c r="L2" s="21"/>
-      <c r="M2" s="21"/>
-      <c r="N2" s="21"/>
-      <c r="O2" s="21"/>
-      <c r="P2" s="21"/>
-      <c r="Q2" s="21"/>
-      <c r="R2" s="21"/>
-      <c r="S2" s="21"/>
-      <c r="T2" s="21"/>
-      <c r="U2" s="21"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="26"/>
+      <c r="I2" s="26"/>
+      <c r="J2" s="26"/>
+      <c r="K2" s="26"/>
+      <c r="L2" s="26"/>
+      <c r="M2" s="26"/>
+      <c r="N2" s="26"/>
+      <c r="O2" s="26"/>
+      <c r="P2" s="26"/>
+      <c r="Q2" s="26"/>
+      <c r="R2" s="26"/>
+      <c r="S2" s="26"/>
+      <c r="T2" s="26"/>
+      <c r="U2" s="26"/>
     </row>
     <row r="3" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B3" s="19"/>
@@ -1400,11 +1394,11 @@
       <c r="R5" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="S5" s="22" t="s">
+      <c r="S5" s="27" t="s">
         <v>106</v>
       </c>
-      <c r="T5" s="22"/>
-      <c r="U5" s="22"/>
+      <c r="T5" s="27"/>
+      <c r="U5" s="27"/>
     </row>
     <row r="6" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -1435,9 +1429,8 @@
       <c r="R6" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="S6" s="2" t="str">
-        <f>"Từ ngày {{TuNgay}}"&amp;" đến ngày {{DenNgay}}"</f>
-        <v>Từ ngày {{TuNgay}} đến ngày {{DenNgay}}</v>
+      <c r="S6" s="2" t="s">
+        <v>107</v>
       </c>
       <c r="T6" s="2"/>
       <c r="U6" s="2"/>
@@ -1466,86 +1459,86 @@
       <c r="U7" s="2"/>
     </row>
     <row r="8" spans="1:21" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A8" s="23" t="s">
+      <c r="A8" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="26" t="s">
+      <c r="B8" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="26" t="s">
+      <c r="C8" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="D8" s="26" t="s">
+      <c r="D8" s="23" t="s">
         <v>61</v>
       </c>
-      <c r="E8" s="27" t="s">
+      <c r="E8" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="F8" s="28"/>
-      <c r="G8" s="28"/>
-      <c r="H8" s="28"/>
-      <c r="I8" s="28"/>
-      <c r="J8" s="28"/>
-      <c r="K8" s="29"/>
-      <c r="L8" s="30" t="s">
+      <c r="F8" s="32"/>
+      <c r="G8" s="32"/>
+      <c r="H8" s="32"/>
+      <c r="I8" s="32"/>
+      <c r="J8" s="32"/>
+      <c r="K8" s="33"/>
+      <c r="L8" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="M8" s="30"/>
-      <c r="N8" s="30"/>
-      <c r="O8" s="30"/>
-      <c r="P8" s="30"/>
-      <c r="Q8" s="30"/>
-      <c r="R8" s="30"/>
-      <c r="S8" s="30"/>
-      <c r="T8" s="30"/>
+      <c r="M8" s="24"/>
+      <c r="N8" s="24"/>
+      <c r="O8" s="24"/>
+      <c r="P8" s="24"/>
+      <c r="Q8" s="24"/>
+      <c r="R8" s="24"/>
+      <c r="S8" s="24"/>
+      <c r="T8" s="24"/>
       <c r="U8" s="13"/>
     </row>
     <row r="9" spans="1:21" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A9" s="24"/>
-      <c r="B9" s="26"/>
-      <c r="C9" s="26"/>
-      <c r="D9" s="26"/>
-      <c r="E9" s="26" t="s">
+      <c r="A9" s="29"/>
+      <c r="B9" s="23"/>
+      <c r="C9" s="23"/>
+      <c r="D9" s="23"/>
+      <c r="E9" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="F9" s="26"/>
-      <c r="G9" s="26"/>
-      <c r="H9" s="26"/>
-      <c r="I9" s="26" t="s">
+      <c r="F9" s="23"/>
+      <c r="G9" s="23"/>
+      <c r="H9" s="23"/>
+      <c r="I9" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="J9" s="26"/>
-      <c r="K9" s="26" t="s">
+      <c r="J9" s="23"/>
+      <c r="K9" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="L9" s="30" t="s">
+      <c r="L9" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="M9" s="30"/>
-      <c r="N9" s="30"/>
-      <c r="O9" s="30"/>
-      <c r="P9" s="26" t="s">
+      <c r="M9" s="24"/>
+      <c r="N9" s="24"/>
+      <c r="O9" s="24"/>
+      <c r="P9" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="Q9" s="26"/>
-      <c r="R9" s="30" t="s">
+      <c r="Q9" s="23"/>
+      <c r="R9" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="S9" s="26" t="s">
+      <c r="S9" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="T9" s="26" t="s">
+      <c r="T9" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="U9" s="26" t="s">
+      <c r="U9" s="23" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:21" ht="45.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="25"/>
-      <c r="B10" s="26"/>
-      <c r="C10" s="26"/>
-      <c r="D10" s="26"/>
+      <c r="A10" s="30"/>
+      <c r="B10" s="23"/>
+      <c r="C10" s="23"/>
+      <c r="D10" s="23"/>
       <c r="E10" s="6" t="s">
         <v>22</v>
       </c>
@@ -1564,7 +1557,7 @@
       <c r="J10" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="K10" s="26"/>
+      <c r="K10" s="23"/>
       <c r="L10" s="6" t="s">
         <v>22</v>
       </c>
@@ -1583,10 +1576,10 @@
       <c r="Q10" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="R10" s="30"/>
-      <c r="S10" s="26"/>
-      <c r="T10" s="26"/>
-      <c r="U10" s="26"/>
+      <c r="R10" s="24"/>
+      <c r="S10" s="23"/>
+      <c r="T10" s="23"/>
+      <c r="U10" s="23"/>
     </row>
     <row r="11" spans="1:21" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A11" s="13" t="s">
@@ -1599,11 +1592,11 @@
         <v>30</v>
       </c>
       <c r="D11" s="18"/>
-      <c r="E11" s="31" t="s">
+      <c r="E11" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="F11" s="32"/>
-      <c r="G11" s="33"/>
+      <c r="F11" s="21"/>
+      <c r="G11" s="22"/>
       <c r="H11" s="6" t="s">
         <v>32</v>
       </c>
@@ -1616,11 +1609,11 @@
       <c r="K11" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="L11" s="31" t="s">
+      <c r="L11" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="M11" s="32"/>
-      <c r="N11" s="33"/>
+      <c r="M11" s="21"/>
+      <c r="N11" s="22"/>
       <c r="O11" s="6" t="s">
         <v>37</v>
       </c>
@@ -2748,11 +2741,6 @@
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="E11:G11"/>
-    <mergeCell ref="L11:N11"/>
-    <mergeCell ref="I9:J9"/>
-    <mergeCell ref="K9:K10"/>
-    <mergeCell ref="L9:O9"/>
     <mergeCell ref="A1:U1"/>
     <mergeCell ref="A2:U2"/>
     <mergeCell ref="S5:U5"/>
@@ -2768,12 +2756,17 @@
     <mergeCell ref="R9:R10"/>
     <mergeCell ref="S9:S10"/>
     <mergeCell ref="D8:D10"/>
+    <mergeCell ref="E11:G11"/>
+    <mergeCell ref="L11:N11"/>
+    <mergeCell ref="I9:J9"/>
+    <mergeCell ref="K9:K10"/>
+    <mergeCell ref="L9:O9"/>
   </mergeCells>
   <conditionalFormatting sqref="A12:U50">
-    <cfRule type="expression" dxfId="2" priority="1">
+    <cfRule type="expression" dxfId="1" priority="1">
       <formula>ISNUMBER($E12)=FALSE</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="0" priority="2">
       <formula>ISNUMBER($A12)</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>